<commit_message>
feat: update KPI logic and add data informe view
</commit_message>
<xml_diff>
--- a/Auditorias_Clientes/Bata/Bata 25/Reporte_Auditoria_Maestro_Bata_Bata_25_Consolidado.xlsx
+++ b/Auditorias_Clientes/Bata/Bata 25/Reporte_Auditoria_Maestro_Bata_Bata_25_Consolidado.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -88,8 +88,12 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -160,6 +164,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F2F2F2"/>
         <bgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001B2A4A"/>
+        <bgColor rgb="001B2A4A"/>
       </patternFill>
     </fill>
   </fills>
@@ -434,7 +444,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -575,6 +585,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="11" fillId="12" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1631,7 +1650,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="16659225" cy="6191250"/>
+    <ext cx="37509450" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -1656,7 +1675,7 @@
       <row>29</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="9020175" cy="6781800"/>
+    <ext cx="19697700" cy="14001750"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -1686,7 +1705,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8534400" cy="6191250"/>
+    <ext cx="17335500" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -1711,7 +1730,7 @@
       <row>26</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="12468225" cy="6191250"/>
+    <ext cx="29965650" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -1736,7 +1755,7 @@
       <row>26</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="12468225" cy="6191250"/>
+    <ext cx="29965650" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="3" name="Image 3" descr="Picture"/>
@@ -1761,7 +1780,7 @@
       <row>54</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8534400" cy="6191250"/>
+    <ext cx="17335500" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="4" name="Image 4" descr="Picture"/>
@@ -1786,7 +1805,7 @@
       <row>79</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6972300" cy="6191250"/>
+    <ext cx="16554450" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="5" name="Image 5" descr="Picture"/>
@@ -1811,7 +1830,7 @@
       <row>79</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7629525" cy="6191250"/>
+    <ext cx="16554450" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="6" name="Image 6" descr="Picture"/>
@@ -1836,7 +1855,7 @@
       <row>107</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8534400" cy="6191250"/>
+    <ext cx="17335500" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="7" name="Image 7" descr="Picture"/>
@@ -1861,7 +1880,7 @@
       <row>132</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="9324975" cy="6191250"/>
+    <ext cx="23050500" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="8" name="Image 8" descr="Picture"/>
@@ -1886,7 +1905,7 @@
       <row>132</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="9324975" cy="6191250"/>
+    <ext cx="23050500" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="9" name="Image 9" descr="Picture"/>
@@ -1911,7 +1930,7 @@
       <row>160</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8534400" cy="6191250"/>
+    <ext cx="17335500" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="10" name="Image 10" descr="Picture"/>
@@ -1936,7 +1955,7 @@
       <row>185</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6972300" cy="6191250"/>
+    <ext cx="16554450" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="11" name="Image 11" descr="Picture"/>
@@ -1961,7 +1980,7 @@
       <row>185</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7629525" cy="6191250"/>
+    <ext cx="16554450" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="12" name="Image 12" descr="Picture"/>
@@ -1991,7 +2010,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6181725" cy="6191250"/>
+    <ext cx="16554450" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -2016,7 +2035,7 @@
       <row>26</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6467475" cy="6191250"/>
+    <ext cx="16554450" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -2041,7 +2060,7 @@
       <row>51</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6229350" cy="6191250"/>
+    <ext cx="16554450" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="3" name="Image 3" descr="Picture"/>
@@ -2066,7 +2085,7 @@
       <row>76</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6219825" cy="6191250"/>
+    <ext cx="16554450" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="4" name="Image 4" descr="Picture"/>
@@ -2091,7 +2110,7 @@
       <row>101</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6591300" cy="6191250"/>
+    <ext cx="16554450" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="5" name="Image 5" descr="Picture"/>
@@ -2116,7 +2135,7 @@
       <row>126</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6562725" cy="6191250"/>
+    <ext cx="16554450" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="6" name="Image 6" descr="Picture"/>
@@ -2141,7 +2160,7 @@
       <row>151</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6200775" cy="6191250"/>
+    <ext cx="16554450" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="7" name="Image 7" descr="Picture"/>
@@ -2166,7 +2185,7 @@
       <row>176</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6181725" cy="6191250"/>
+    <ext cx="16554450" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="8" name="Image 8" descr="Picture"/>
@@ -2191,7 +2210,7 @@
       <row>201</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7058025" cy="6191250"/>
+    <ext cx="16554450" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="9" name="Image 9" descr="Picture"/>
@@ -2216,7 +2235,7 @@
       <row>226</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6467475" cy="6191250"/>
+    <ext cx="16554450" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="10" name="Image 10" descr="Picture"/>
@@ -2241,7 +2260,7 @@
       <row>251</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6467475" cy="6191250"/>
+    <ext cx="16554450" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="11" name="Image 11" descr="Picture"/>
@@ -2266,7 +2285,7 @@
       <row>276</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7105650" cy="6191250"/>
+    <ext cx="16554450" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="12" name="Image 12" descr="Picture"/>
@@ -2291,7 +2310,7 @@
       <row>301</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6200775" cy="6191250"/>
+    <ext cx="16554450" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="13" name="Image 13" descr="Picture"/>
@@ -2321,7 +2340,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6048375" cy="6181725"/>
+    <ext cx="16554450" cy="14049375"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -2346,7 +2365,7 @@
       <row>27</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6048375" cy="6191250"/>
+    <ext cx="16554450" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -2371,7 +2390,7 @@
       <row>52</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6048375" cy="6191250"/>
+    <ext cx="16554450" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="3" name="Image 3" descr="Picture"/>
@@ -2396,7 +2415,7 @@
       <row>77</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6048375" cy="6191250"/>
+    <ext cx="16554450" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="4" name="Image 4" descr="Picture"/>
@@ -2421,7 +2440,7 @@
       <row>102</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6048375" cy="6191250"/>
+    <ext cx="16554450" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="5" name="Image 5" descr="Picture"/>
@@ -2446,7 +2465,7 @@
       <row>127</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6048375" cy="6191250"/>
+    <ext cx="16554450" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="6" name="Image 6" descr="Picture"/>
@@ -2471,7 +2490,7 @@
       <row>152</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6048375" cy="6191250"/>
+    <ext cx="16554450" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="7" name="Image 7" descr="Picture"/>
@@ -2496,7 +2515,7 @@
       <row>177</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6048375" cy="6191250"/>
+    <ext cx="16554450" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="8" name="Image 8" descr="Picture"/>
@@ -2521,7 +2540,7 @@
       <row>202</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6048375" cy="6191250"/>
+    <ext cx="16554450" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="9" name="Image 9" descr="Picture"/>
@@ -2546,7 +2565,7 @@
       <row>227</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6048375" cy="6191250"/>
+    <ext cx="16554450" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="10" name="Image 10" descr="Picture"/>
@@ -2571,7 +2590,7 @@
       <row>252</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6048375" cy="6191250"/>
+    <ext cx="16554450" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="11" name="Image 11" descr="Picture"/>
@@ -2596,7 +2615,7 @@
       <row>277</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6048375" cy="6191250"/>
+    <ext cx="16554450" cy="14058900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="12" name="Image 12" descr="Picture"/>
@@ -2604,56 +2623,6 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId12"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>302</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="6048375" cy="6191250"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="13" name="Image 13" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId13"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>327</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="6048375" cy="6191250"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="14" name="Image 14" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId14"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3040,12 +3009,12 @@
       </c>
       <c r="C2" s="44" t="inlineStr">
         <is>
-          <t>Hora inicio (UTC 0)</t>
+          <t>Hora_inicio</t>
         </is>
       </c>
       <c r="D2" s="44" t="inlineStr">
         <is>
-          <t>Hora término</t>
+          <t>Hora_termino</t>
         </is>
       </c>
       <c r="E2" s="44" t="inlineStr">
@@ -3085,22 +3054,22 @@
       </c>
       <c r="L2" s="44" t="inlineStr">
         <is>
+          <t>% Precisión de Eventos</t>
+        </is>
+      </c>
+      <c r="M2" s="44" t="inlineStr">
+        <is>
           <t>% Eventos Correctos sobre Registrados</t>
         </is>
       </c>
-      <c r="M2" s="44" t="inlineStr">
-        <is>
-          <t>% Eventos Correctos sobre Total</t>
-        </is>
-      </c>
       <c r="N2" s="44" t="inlineStr">
         <is>
-          <t>Eventos Reg. Mal (Sist.)</t>
+          <t>Eventos Malos del Sistema</t>
         </is>
       </c>
       <c r="O2" s="44" t="inlineStr">
         <is>
-          <t>% Eventos Reg. Mal sobre Registrados</t>
+          <t>% Eventos Malos sobre Total</t>
         </is>
       </c>
       <c r="P2" s="44" t="inlineStr">
@@ -3135,12 +3104,12 @@
       </c>
       <c r="V2" s="44" t="inlineStr">
         <is>
-          <t>Precision de Género</t>
+          <t>Precisión de Género</t>
         </is>
       </c>
       <c r="W2" s="44" t="inlineStr">
         <is>
-          <t>% Precision de Género</t>
+          <t>% Precisión de Género</t>
         </is>
       </c>
       <c r="X2" s="44" t="inlineStr">
@@ -3293,68 +3262,44 @@
         <v>62</v>
       </c>
       <c r="G4" s="47" t="n">
-        <v>27</v>
+        <v>58</v>
       </c>
       <c r="H4" s="48" t="n">
-        <v>0.4354838709677419</v>
+        <v>0.9354838709677419</v>
       </c>
       <c r="I4" s="47" t="n">
-        <v>35</v>
+        <v>4</v>
       </c>
       <c r="J4" s="48" t="n">
-        <v>0.5645161290322581</v>
+        <v>0.06451612903225806</v>
       </c>
       <c r="K4" s="47" t="n">
-        <v>27</v>
+        <v>58</v>
       </c>
       <c r="L4" s="48" t="n">
+        <v>0.9354838709677419</v>
+      </c>
+      <c r="M4" s="48" t="n">
         <v>1</v>
       </c>
-      <c r="M4" s="48" t="n">
-        <v>0.4354838709677419</v>
-      </c>
       <c r="N4" s="47" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="O4" s="48" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" s="47" t="n">
-        <v>27</v>
-      </c>
-      <c r="Q4" s="48" t="n">
-        <v>1</v>
-      </c>
-      <c r="R4" s="47" t="n">
-        <v>0</v>
-      </c>
-      <c r="S4" s="48" t="n">
-        <v>0</v>
-      </c>
-      <c r="T4" s="47" t="n">
-        <v>27</v>
-      </c>
-      <c r="U4" s="48" t="n">
-        <v>1</v>
-      </c>
-      <c r="V4" s="47" t="n">
-        <v>25</v>
-      </c>
-      <c r="W4" s="48" t="n">
-        <v>0.9259259259259259</v>
-      </c>
-      <c r="X4" s="47" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y4" s="48" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z4" s="47" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA4" s="48" t="n">
-        <v>0</v>
-      </c>
+        <v>0.06451612903225806</v>
+      </c>
+      <c r="P4" s="47" t="n"/>
+      <c r="Q4" s="48" t="n"/>
+      <c r="R4" s="47" t="n"/>
+      <c r="S4" s="48" t="n"/>
+      <c r="T4" s="47" t="n"/>
+      <c r="U4" s="48" t="n"/>
+      <c r="V4" s="47" t="n"/>
+      <c r="W4" s="48" t="n"/>
+      <c r="X4" s="47" t="n"/>
+      <c r="Y4" s="48" t="n"/>
+      <c r="Z4" s="47" t="n"/>
+      <c r="AA4" s="48" t="n"/>
       <c r="AB4" s="46" t="inlineStr">
         <is>
           <t>Linea_conteo</t>
@@ -3389,25 +3334,25 @@
         <v>50</v>
       </c>
       <c r="G5" s="47" t="n">
-        <v>29</v>
+        <v>50</v>
       </c>
       <c r="H5" s="48" t="n">
-        <v>0.58</v>
+        <v>1</v>
       </c>
       <c r="I5" s="47" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="J5" s="48" t="n">
-        <v>0.42</v>
+        <v>0</v>
       </c>
       <c r="K5" s="47" t="n">
-        <v>29</v>
+        <v>50</v>
       </c>
       <c r="L5" s="48" t="n">
         <v>1</v>
       </c>
       <c r="M5" s="48" t="n">
-        <v>0.58</v>
+        <v>1</v>
       </c>
       <c r="N5" s="47" t="n">
         <v>0</v>
@@ -3415,42 +3360,18 @@
       <c r="O5" s="48" t="n">
         <v>0</v>
       </c>
-      <c r="P5" s="47" t="n">
-        <v>29</v>
-      </c>
-      <c r="Q5" s="48" t="n">
-        <v>1</v>
-      </c>
-      <c r="R5" s="47" t="n">
-        <v>0</v>
-      </c>
-      <c r="S5" s="48" t="n">
-        <v>0</v>
-      </c>
-      <c r="T5" s="47" t="n">
-        <v>29</v>
-      </c>
-      <c r="U5" s="48" t="n">
-        <v>1</v>
-      </c>
-      <c r="V5" s="47" t="n">
-        <v>28</v>
-      </c>
-      <c r="W5" s="48" t="n">
-        <v>0.9655172413793104</v>
-      </c>
-      <c r="X5" s="47" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y5" s="48" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z5" s="47" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA5" s="48" t="n">
-        <v>0</v>
-      </c>
+      <c r="P5" s="47" t="n"/>
+      <c r="Q5" s="48" t="n"/>
+      <c r="R5" s="47" t="n"/>
+      <c r="S5" s="48" t="n"/>
+      <c r="T5" s="47" t="n"/>
+      <c r="U5" s="48" t="n"/>
+      <c r="V5" s="47" t="n"/>
+      <c r="W5" s="48" t="n"/>
+      <c r="X5" s="47" t="n"/>
+      <c r="Y5" s="48" t="n"/>
+      <c r="Z5" s="47" t="n"/>
+      <c r="AA5" s="48" t="n"/>
       <c r="AB5" s="46" t="inlineStr">
         <is>
           <t>Linea_conteo</t>
@@ -3869,34 +3790,34 @@
         <v>11</v>
       </c>
       <c r="G10" s="47" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H10" s="48" t="n">
-        <v>0.9090909090909091</v>
+        <v>1</v>
       </c>
       <c r="I10" s="47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J10" s="48" t="n">
-        <v>0.09090909090909091</v>
+        <v>0</v>
       </c>
       <c r="K10" s="47" t="n">
         <v>10</v>
       </c>
       <c r="L10" s="48" t="n">
-        <v>1</v>
+        <v>0.9090909090909091</v>
       </c>
       <c r="M10" s="48" t="n">
         <v>0.9090909090909091</v>
       </c>
       <c r="N10" s="47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O10" s="48" t="n">
-        <v>0</v>
+        <v>0.09090909090909091</v>
       </c>
       <c r="P10" s="47" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q10" s="48" t="n">
         <v>1</v>
@@ -3911,7 +3832,7 @@
         <v>10</v>
       </c>
       <c r="U10" s="48" t="n">
-        <v>1</v>
+        <v>0.9090909090909091</v>
       </c>
       <c r="V10" s="47" t="n">
         <v>10</v>
@@ -4157,34 +4078,34 @@
         <v>10</v>
       </c>
       <c r="G13" s="47" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H13" s="48" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="I13" s="47" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J13" s="48" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="K13" s="47" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L13" s="48" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="M13" s="48" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="N13" s="47" t="n">
         <v>1</v>
       </c>
-      <c r="M13" s="48" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="N13" s="47" t="n">
-        <v>0</v>
-      </c>
       <c r="O13" s="48" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="P13" s="47" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q13" s="48" t="n">
         <v>1</v>
@@ -4199,7 +4120,7 @@
         <v>8</v>
       </c>
       <c r="U13" s="48" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="V13" s="47" t="n">
         <v>7</v>
@@ -4253,68 +4174,44 @@
         <v>43</v>
       </c>
       <c r="G14" s="47" t="n">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="H14" s="48" t="n">
-        <v>0.6046511627906976</v>
+        <v>0.9302325581395349</v>
       </c>
       <c r="I14" s="47" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="J14" s="48" t="n">
-        <v>0.3953488372093023</v>
+        <v>0.06976744186046512</v>
       </c>
       <c r="K14" s="47" t="n">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="L14" s="48" t="n">
+        <v>0.9302325581395349</v>
+      </c>
+      <c r="M14" s="48" t="n">
         <v>1</v>
       </c>
-      <c r="M14" s="48" t="n">
-        <v>0.6046511627906976</v>
-      </c>
       <c r="N14" s="47" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O14" s="48" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" s="47" t="n">
-        <v>26</v>
-      </c>
-      <c r="Q14" s="48" t="n">
-        <v>1</v>
-      </c>
-      <c r="R14" s="47" t="n">
-        <v>0</v>
-      </c>
-      <c r="S14" s="48" t="n">
-        <v>0</v>
-      </c>
-      <c r="T14" s="47" t="n">
-        <v>26</v>
-      </c>
-      <c r="U14" s="48" t="n">
-        <v>1</v>
-      </c>
-      <c r="V14" s="47" t="n">
-        <v>24</v>
-      </c>
-      <c r="W14" s="48" t="n">
-        <v>0.9230769230769231</v>
-      </c>
-      <c r="X14" s="47" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y14" s="48" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z14" s="47" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA14" s="48" t="n">
-        <v>0</v>
-      </c>
+        <v>0.06976744186046512</v>
+      </c>
+      <c r="P14" s="47" t="n"/>
+      <c r="Q14" s="48" t="n"/>
+      <c r="R14" s="47" t="n"/>
+      <c r="S14" s="48" t="n"/>
+      <c r="T14" s="47" t="n"/>
+      <c r="U14" s="48" t="n"/>
+      <c r="V14" s="47" t="n"/>
+      <c r="W14" s="48" t="n"/>
+      <c r="X14" s="47" t="n"/>
+      <c r="Y14" s="48" t="n"/>
+      <c r="Z14" s="47" t="n"/>
+      <c r="AA14" s="48" t="n"/>
       <c r="AB14" s="46" t="inlineStr">
         <is>
           <t>Linea_conteo</t>
@@ -4349,68 +4246,44 @@
         <v>53</v>
       </c>
       <c r="G15" s="47" t="n">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="H15" s="48" t="n">
-        <v>0.6037735849056604</v>
+        <v>0.9622641509433962</v>
       </c>
       <c r="I15" s="47" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="J15" s="48" t="n">
-        <v>0.3962264150943396</v>
+        <v>0.03773584905660377</v>
       </c>
       <c r="K15" s="47" t="n">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="L15" s="48" t="n">
-        <v>1</v>
+        <v>0.9433962264150944</v>
       </c>
       <c r="M15" s="48" t="n">
-        <v>0.6037735849056604</v>
+        <v>0.9803921568627451</v>
       </c>
       <c r="N15" s="47" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O15" s="48" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" s="47" t="n">
-        <v>32</v>
-      </c>
-      <c r="Q15" s="48" t="n">
-        <v>1</v>
-      </c>
-      <c r="R15" s="47" t="n">
-        <v>0</v>
-      </c>
-      <c r="S15" s="48" t="n">
-        <v>0</v>
-      </c>
-      <c r="T15" s="47" t="n">
-        <v>32</v>
-      </c>
-      <c r="U15" s="48" t="n">
-        <v>1</v>
-      </c>
-      <c r="V15" s="47" t="n">
-        <v>31</v>
-      </c>
-      <c r="W15" s="48" t="n">
-        <v>0.96875</v>
-      </c>
-      <c r="X15" s="47" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y15" s="48" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z15" s="47" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA15" s="48" t="n">
-        <v>0</v>
-      </c>
+        <v>0.05660377358490566</v>
+      </c>
+      <c r="P15" s="47" t="n"/>
+      <c r="Q15" s="48" t="n"/>
+      <c r="R15" s="47" t="n"/>
+      <c r="S15" s="48" t="n"/>
+      <c r="T15" s="47" t="n"/>
+      <c r="U15" s="48" t="n"/>
+      <c r="V15" s="47" t="n"/>
+      <c r="W15" s="48" t="n"/>
+      <c r="X15" s="47" t="n"/>
+      <c r="Y15" s="48" t="n"/>
+      <c r="Z15" s="47" t="n"/>
+      <c r="AA15" s="48" t="n"/>
       <c r="AB15" s="46" t="inlineStr">
         <is>
           <t>Linea_conteo</t>
@@ -5789,34 +5662,34 @@
         <v>39</v>
       </c>
       <c r="G30" s="47" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="H30" s="48" t="n">
-        <v>0.8461538461538461</v>
+        <v>1</v>
       </c>
       <c r="I30" s="47" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J30" s="48" t="n">
-        <v>0.1538461538461539</v>
+        <v>0</v>
       </c>
       <c r="K30" s="47" t="n">
         <v>33</v>
       </c>
       <c r="L30" s="48" t="n">
-        <v>1</v>
+        <v>0.8461538461538461</v>
       </c>
       <c r="M30" s="48" t="n">
         <v>0.8461538461538461</v>
       </c>
       <c r="N30" s="47" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="O30" s="48" t="n">
-        <v>0</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="P30" s="47" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="Q30" s="48" t="n">
         <v>1</v>
@@ -5831,7 +5704,7 @@
         <v>33</v>
       </c>
       <c r="U30" s="48" t="n">
-        <v>1</v>
+        <v>0.8461538461538461</v>
       </c>
       <c r="V30" s="47" t="n">
         <v>33</v>
@@ -5885,34 +5758,34 @@
         <v>32</v>
       </c>
       <c r="G31" s="47" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H31" s="48" t="n">
-        <v>0.9375</v>
+        <v>1</v>
       </c>
       <c r="I31" s="47" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J31" s="48" t="n">
-        <v>0.0625</v>
+        <v>0</v>
       </c>
       <c r="K31" s="47" t="n">
         <v>30</v>
       </c>
       <c r="L31" s="48" t="n">
-        <v>1</v>
+        <v>0.9375</v>
       </c>
       <c r="M31" s="48" t="n">
         <v>0.9375</v>
       </c>
       <c r="N31" s="47" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O31" s="48" t="n">
-        <v>0</v>
+        <v>0.0625</v>
       </c>
       <c r="P31" s="47" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="Q31" s="48" t="n">
         <v>1</v>
@@ -5927,7 +5800,7 @@
         <v>30</v>
       </c>
       <c r="U31" s="48" t="n">
-        <v>1</v>
+        <v>0.9375</v>
       </c>
       <c r="V31" s="47" t="n">
         <v>28</v>
@@ -6255,34 +6128,34 @@
         <v>626</v>
       </c>
       <c r="G35" s="50" t="n">
-        <v>521</v>
+        <v>617</v>
       </c>
       <c r="H35" s="51" t="n">
-        <v>0.8322683706070287</v>
+        <v>0.9856230031948882</v>
       </c>
       <c r="I35" s="50" t="n">
-        <v>105</v>
+        <v>9</v>
       </c>
       <c r="J35" s="51" t="n">
-        <v>0.1677316293929713</v>
+        <v>0.01437699680511182</v>
       </c>
       <c r="K35" s="50" t="n">
-        <v>520</v>
+        <v>605</v>
       </c>
       <c r="L35" s="51" t="n">
-        <v>0.9980806142034548</v>
+        <v>0.9664536741214057</v>
       </c>
       <c r="M35" s="51" t="n">
-        <v>0.8306709265175719</v>
+        <v>0.9805510534846029</v>
       </c>
       <c r="N35" s="50" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="O35" s="51" t="n">
-        <v>0.001919385796545105</v>
+        <v>0.03354632587859425</v>
       </c>
       <c r="P35" s="50" t="n">
-        <v>521</v>
+        <v>418</v>
       </c>
       <c r="Q35" s="51" t="n">
         <v>1</v>
@@ -6294,16 +6167,16 @@
         <v>0</v>
       </c>
       <c r="T35" s="50" t="n">
-        <v>521</v>
+        <v>407</v>
       </c>
       <c r="U35" s="51" t="n">
-        <v>1</v>
+        <v>0.9736842105263158</v>
       </c>
       <c r="V35" s="50" t="n">
-        <v>497</v>
+        <v>389</v>
       </c>
       <c r="W35" s="51" t="n">
-        <v>0.9539347408829175</v>
+        <v>0.9557739557739557</v>
       </c>
       <c r="X35" s="50" t="n">
         <v>0</v>
@@ -33224,9 +33097,1394 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="L2:AM31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="2">
+      <c r="L2" s="52" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="M2" s="52" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="N2" s="52" t="inlineStr">
+        <is>
+          <t>Hora_inicio</t>
+        </is>
+      </c>
+      <c r="O2" s="52" t="inlineStr">
+        <is>
+          <t>Hora_termino</t>
+        </is>
+      </c>
+      <c r="P2" s="52" t="inlineStr">
+        <is>
+          <t>Cámara</t>
+        </is>
+      </c>
+      <c r="Q2" s="52" t="inlineStr">
+        <is>
+          <t>Total Eventos</t>
+        </is>
+      </c>
+      <c r="R2" s="52" t="inlineStr">
+        <is>
+          <t>Eventos Registrados por el Sistema</t>
+        </is>
+      </c>
+      <c r="S2" s="52" t="inlineStr">
+        <is>
+          <t>% Eventos Registrados por el Sistema</t>
+        </is>
+      </c>
+      <c r="T2" s="52" t="inlineStr">
+        <is>
+          <t>Eventos NO Registrados (Manuales)</t>
+        </is>
+      </c>
+      <c r="U2" s="52" t="inlineStr">
+        <is>
+          <t>% Eventos NO Registrados (Manuales)</t>
+        </is>
+      </c>
+      <c r="V2" s="52" t="inlineStr">
+        <is>
+          <t>Eventos Correctos del Sistema</t>
+        </is>
+      </c>
+      <c r="W2" s="52" t="inlineStr">
+        <is>
+          <t>% Precisión de Eventos</t>
+        </is>
+      </c>
+      <c r="X2" s="52" t="inlineStr">
+        <is>
+          <t>% Eventos Correctos sobre Registrados</t>
+        </is>
+      </c>
+      <c r="Y2" s="52" t="inlineStr">
+        <is>
+          <t>Eventos Malos del Sistema</t>
+        </is>
+      </c>
+      <c r="Z2" s="52" t="inlineStr">
+        <is>
+          <t>% Eventos Malos sobre Total</t>
+        </is>
+      </c>
+      <c r="AA2" s="52" t="inlineStr">
+        <is>
+          <t>Cobertura Identity</t>
+        </is>
+      </c>
+      <c r="AB2" s="52" t="inlineStr">
+        <is>
+          <t>% Cobertura Identity</t>
+        </is>
+      </c>
+      <c r="AC2" s="52" t="inlineStr">
+        <is>
+          <t>Identity Unknown</t>
+        </is>
+      </c>
+      <c r="AD2" s="52" t="inlineStr">
+        <is>
+          <t>% Identity Unknown</t>
+        </is>
+      </c>
+      <c r="AE2" s="52" t="inlineStr">
+        <is>
+          <t>Cobertura Género</t>
+        </is>
+      </c>
+      <c r="AF2" s="52" t="inlineStr">
+        <is>
+          <t>% Cobertura Género</t>
+        </is>
+      </c>
+      <c r="AG2" s="52" t="inlineStr">
+        <is>
+          <t>Precisión de Género</t>
+        </is>
+      </c>
+      <c r="AH2" s="52" t="inlineStr">
+        <is>
+          <t>% Precisión de Género</t>
+        </is>
+      </c>
+      <c r="AI2" s="52" t="inlineStr">
+        <is>
+          <t>Cobertura Edad</t>
+        </is>
+      </c>
+      <c r="AJ2" s="52" t="inlineStr">
+        <is>
+          <t>% Cobertura Edad</t>
+        </is>
+      </c>
+      <c r="AK2" s="52" t="inlineStr">
+        <is>
+          <t>Precisión de Edad</t>
+        </is>
+      </c>
+      <c r="AL2" s="52" t="inlineStr">
+        <is>
+          <t>% Precisión de Edad</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="L3" s="53" t="inlineStr">
+        <is>
+          <t>Entrada</t>
+        </is>
+      </c>
+      <c r="M3" s="53" t="inlineStr"/>
+      <c r="N3" s="53" t="inlineStr"/>
+      <c r="O3" s="53" t="inlineStr"/>
+      <c r="P3" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q3" s="53" t="n">
+        <v>18</v>
+      </c>
+      <c r="R3" s="53" t="n">
+        <v>18</v>
+      </c>
+      <c r="S3" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="T3" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="V3" s="53" t="n">
+        <v>17</v>
+      </c>
+      <c r="W3" s="54" t="n">
+        <v>0.9444444444444444</v>
+      </c>
+      <c r="X3" s="54" t="n">
+        <v>0.9444444444444444</v>
+      </c>
+      <c r="Y3" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z3" s="54" t="n">
+        <v>0.05555555555555555</v>
+      </c>
+      <c r="AA3" s="53" t="n">
+        <v>18</v>
+      </c>
+      <c r="AB3" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC3" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD3" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE3" s="53" t="n">
+        <v>16</v>
+      </c>
+      <c r="AF3" s="54" t="n">
+        <v>0.8888888888888888</v>
+      </c>
+      <c r="AG3" s="53" t="n">
+        <v>14</v>
+      </c>
+      <c r="AH3" s="54" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="AI3" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ3" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK3" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL3" s="54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="L4" s="53" t="inlineStr">
+        <is>
+          <t>Exploracion 1</t>
+        </is>
+      </c>
+      <c r="M4" s="53" t="inlineStr"/>
+      <c r="N4" s="53" t="inlineStr"/>
+      <c r="O4" s="53" t="inlineStr"/>
+      <c r="P4" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q4" s="53" t="n">
+        <v>30</v>
+      </c>
+      <c r="R4" s="53" t="n">
+        <v>30</v>
+      </c>
+      <c r="S4" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="T4" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="U4" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="V4" s="53" t="n">
+        <v>30</v>
+      </c>
+      <c r="W4" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="X4" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y4" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z4" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA4" s="53" t="n">
+        <v>30</v>
+      </c>
+      <c r="AB4" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC4" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD4" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE4" s="53" t="n">
+        <v>30</v>
+      </c>
+      <c r="AF4" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG4" s="53" t="n">
+        <v>29</v>
+      </c>
+      <c r="AH4" s="54" t="n">
+        <v>0.9666666666666667</v>
+      </c>
+      <c r="AI4" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ4" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK4" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL4" s="54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="L5" s="53" t="inlineStr">
+        <is>
+          <t>Exterior 2</t>
+        </is>
+      </c>
+      <c r="M5" s="53" t="inlineStr"/>
+      <c r="N5" s="53" t="inlineStr"/>
+      <c r="O5" s="53" t="inlineStr"/>
+      <c r="P5" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q5" s="53" t="n">
+        <v>105</v>
+      </c>
+      <c r="R5" s="53" t="n">
+        <v>98</v>
+      </c>
+      <c r="S5" s="54" t="n">
+        <v>0.9333333333333333</v>
+      </c>
+      <c r="T5" s="53" t="n">
+        <v>7</v>
+      </c>
+      <c r="U5" s="54" t="n">
+        <v>0.06666666666666667</v>
+      </c>
+      <c r="V5" s="53" t="n">
+        <v>98</v>
+      </c>
+      <c r="W5" s="54" t="n">
+        <v>0.9333333333333333</v>
+      </c>
+      <c r="X5" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y5" s="53" t="n">
+        <v>7</v>
+      </c>
+      <c r="Z5" s="54" t="n">
+        <v>0.06666666666666667</v>
+      </c>
+      <c r="AA5" s="53" t="n">
+        <v/>
+      </c>
+      <c r="AB5" s="54" t="n">
+        <v/>
+      </c>
+      <c r="AC5" s="53" t="n">
+        <v/>
+      </c>
+      <c r="AD5" s="54" t="n">
+        <v/>
+      </c>
+      <c r="AE5" s="53" t="n">
+        <v/>
+      </c>
+      <c r="AF5" s="54" t="n">
+        <v/>
+      </c>
+      <c r="AG5" s="53" t="n">
+        <v/>
+      </c>
+      <c r="AH5" s="54" t="n">
+        <v/>
+      </c>
+      <c r="AI5" s="53" t="n">
+        <v/>
+      </c>
+      <c r="AJ5" s="54" t="n">
+        <v/>
+      </c>
+      <c r="AK5" s="53" t="n">
+        <v/>
+      </c>
+      <c r="AL5" s="54" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="L6" s="53" t="inlineStr">
+        <is>
+          <t>Exterior L</t>
+        </is>
+      </c>
+      <c r="M6" s="53" t="inlineStr"/>
+      <c r="N6" s="53" t="inlineStr"/>
+      <c r="O6" s="53" t="inlineStr"/>
+      <c r="P6" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q6" s="53" t="n">
+        <v>103</v>
+      </c>
+      <c r="R6" s="53" t="n">
+        <v>101</v>
+      </c>
+      <c r="S6" s="54" t="n">
+        <v>0.9805825242718447</v>
+      </c>
+      <c r="T6" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="U6" s="54" t="n">
+        <v>0.01941747572815534</v>
+      </c>
+      <c r="V6" s="53" t="n">
+        <v>100</v>
+      </c>
+      <c r="W6" s="54" t="n">
+        <v>0.970873786407767</v>
+      </c>
+      <c r="X6" s="54" t="n">
+        <v>0.9900990099009901</v>
+      </c>
+      <c r="Y6" s="53" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z6" s="54" t="n">
+        <v>0.02912621359223301</v>
+      </c>
+      <c r="AA6" s="53" t="n">
+        <v/>
+      </c>
+      <c r="AB6" s="54" t="n">
+        <v/>
+      </c>
+      <c r="AC6" s="53" t="n">
+        <v/>
+      </c>
+      <c r="AD6" s="54" t="n">
+        <v/>
+      </c>
+      <c r="AE6" s="53" t="n">
+        <v/>
+      </c>
+      <c r="AF6" s="54" t="n">
+        <v/>
+      </c>
+      <c r="AG6" s="53" t="n">
+        <v/>
+      </c>
+      <c r="AH6" s="54" t="n">
+        <v/>
+      </c>
+      <c r="AI6" s="53" t="n">
+        <v/>
+      </c>
+      <c r="AJ6" s="54" t="n">
+        <v/>
+      </c>
+      <c r="AK6" s="53" t="n">
+        <v/>
+      </c>
+      <c r="AL6" s="54" t="n">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="L7" s="53" t="inlineStr">
+        <is>
+          <t>Vitrina Exterior</t>
+        </is>
+      </c>
+      <c r="M7" s="53" t="inlineStr"/>
+      <c r="N7" s="53" t="inlineStr"/>
+      <c r="O7" s="53" t="inlineStr"/>
+      <c r="P7" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q7" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="R7" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="S7" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="T7" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="V7" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="W7" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="X7" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y7" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z7" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA7" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB7" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC7" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD7" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE7" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="AF7" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG7" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="AH7" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI7" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ7" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK7" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL7" s="54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="L8" s="53" t="inlineStr">
+        <is>
+          <t>Vitrina Interior</t>
+        </is>
+      </c>
+      <c r="M8" s="53" t="inlineStr"/>
+      <c r="N8" s="53" t="inlineStr"/>
+      <c r="O8" s="53" t="inlineStr"/>
+      <c r="P8" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="53" t="n">
+        <v>14</v>
+      </c>
+      <c r="R8" s="53" t="n">
+        <v>14</v>
+      </c>
+      <c r="S8" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="T8" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="V8" s="53" t="n">
+        <v>14</v>
+      </c>
+      <c r="W8" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="X8" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y8" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z8" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA8" s="53" t="n">
+        <v>14</v>
+      </c>
+      <c r="AB8" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC8" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD8" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE8" s="53" t="n">
+        <v>14</v>
+      </c>
+      <c r="AF8" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG8" s="53" t="n">
+        <v>14</v>
+      </c>
+      <c r="AH8" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI8" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ8" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK8" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL8" s="54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="L9" s="53" t="inlineStr">
+        <is>
+          <t>Interior 1</t>
+        </is>
+      </c>
+      <c r="M9" s="53" t="inlineStr"/>
+      <c r="N9" s="53" t="inlineStr"/>
+      <c r="O9" s="53" t="inlineStr"/>
+      <c r="P9" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q9" s="53" t="n">
+        <v>16</v>
+      </c>
+      <c r="R9" s="53" t="n">
+        <v>16</v>
+      </c>
+      <c r="S9" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="T9" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="V9" s="53" t="n">
+        <v>16</v>
+      </c>
+      <c r="W9" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="X9" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y9" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z9" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA9" s="53" t="n">
+        <v>16</v>
+      </c>
+      <c r="AB9" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC9" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD9" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE9" s="53" t="n">
+        <v>16</v>
+      </c>
+      <c r="AF9" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG9" s="53" t="n">
+        <v>12</v>
+      </c>
+      <c r="AH9" s="54" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AI9" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ9" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK9" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL9" s="54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="L10" s="53" t="inlineStr">
+        <is>
+          <t>Caja</t>
+        </is>
+      </c>
+      <c r="M10" s="53" t="inlineStr"/>
+      <c r="N10" s="53" t="inlineStr"/>
+      <c r="O10" s="53" t="inlineStr"/>
+      <c r="P10" s="53" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q10" s="53" t="n">
+        <v>77</v>
+      </c>
+      <c r="R10" s="53" t="n">
+        <v>77</v>
+      </c>
+      <c r="S10" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="T10" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="U10" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="V10" s="53" t="n">
+        <v>77</v>
+      </c>
+      <c r="W10" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="X10" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y10" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z10" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA10" s="53" t="n">
+        <v>77</v>
+      </c>
+      <c r="AB10" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC10" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD10" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE10" s="53" t="n">
+        <v>77</v>
+      </c>
+      <c r="AF10" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG10" s="53" t="n">
+        <v>73</v>
+      </c>
+      <c r="AH10" s="54" t="n">
+        <v>0.948051948051948</v>
+      </c>
+      <c r="AI10" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ10" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK10" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL10" s="54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="L11" s="53" t="inlineStr">
+        <is>
+          <t>Estanteria Principal</t>
+        </is>
+      </c>
+      <c r="M11" s="53" t="inlineStr"/>
+      <c r="N11" s="53" t="inlineStr"/>
+      <c r="O11" s="53" t="inlineStr"/>
+      <c r="P11" s="53" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q11" s="53" t="n">
+        <v>106</v>
+      </c>
+      <c r="R11" s="53" t="n">
+        <v>106</v>
+      </c>
+      <c r="S11" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="T11" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="V11" s="53" t="n">
+        <v>100</v>
+      </c>
+      <c r="W11" s="54" t="n">
+        <v>0.9433962264150944</v>
+      </c>
+      <c r="X11" s="54" t="n">
+        <v>0.9433962264150944</v>
+      </c>
+      <c r="Y11" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z11" s="54" t="n">
+        <v>0.05660377358490566</v>
+      </c>
+      <c r="AA11" s="53" t="n">
+        <v>106</v>
+      </c>
+      <c r="AB11" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC11" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD11" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE11" s="53" t="n">
+        <v>100</v>
+      </c>
+      <c r="AF11" s="54" t="n">
+        <v>0.9433962264150944</v>
+      </c>
+      <c r="AG11" s="53" t="n">
+        <v>100</v>
+      </c>
+      <c r="AH11" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI11" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ11" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK11" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL11" s="54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="L12" s="53" t="inlineStr">
+        <is>
+          <t>Exploracion 2</t>
+        </is>
+      </c>
+      <c r="M12" s="53" t="inlineStr"/>
+      <c r="N12" s="53" t="inlineStr"/>
+      <c r="O12" s="53" t="inlineStr"/>
+      <c r="P12" s="53" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q12" s="53" t="n">
+        <v>56</v>
+      </c>
+      <c r="R12" s="53" t="n">
+        <v>56</v>
+      </c>
+      <c r="S12" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="T12" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="V12" s="53" t="n">
+        <v>53</v>
+      </c>
+      <c r="W12" s="54" t="n">
+        <v>0.9464285714285714</v>
+      </c>
+      <c r="X12" s="54" t="n">
+        <v>0.9464285714285714</v>
+      </c>
+      <c r="Y12" s="53" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z12" s="54" t="n">
+        <v>0.05357142857142857</v>
+      </c>
+      <c r="AA12" s="53" t="n">
+        <v>56</v>
+      </c>
+      <c r="AB12" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC12" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD12" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE12" s="53" t="n">
+        <v>53</v>
+      </c>
+      <c r="AF12" s="54" t="n">
+        <v>0.9464285714285714</v>
+      </c>
+      <c r="AG12" s="53" t="n">
+        <v>50</v>
+      </c>
+      <c r="AH12" s="54" t="n">
+        <v>0.9433962264150944</v>
+      </c>
+      <c r="AI12" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ12" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK12" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL12" s="54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="L13" s="53" t="inlineStr">
+        <is>
+          <t>Exploracion 3</t>
+        </is>
+      </c>
+      <c r="M13" s="53" t="inlineStr"/>
+      <c r="N13" s="53" t="inlineStr"/>
+      <c r="O13" s="53" t="inlineStr"/>
+      <c r="P13" s="53" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q13" s="53" t="n">
+        <v>32</v>
+      </c>
+      <c r="R13" s="53" t="n">
+        <v>32</v>
+      </c>
+      <c r="S13" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="T13" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="U13" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="V13" s="53" t="n">
+        <v>31</v>
+      </c>
+      <c r="W13" s="54" t="n">
+        <v>0.96875</v>
+      </c>
+      <c r="X13" s="54" t="n">
+        <v>0.96875</v>
+      </c>
+      <c r="Y13" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z13" s="54" t="n">
+        <v>0.03125</v>
+      </c>
+      <c r="AA13" s="53" t="n">
+        <v>32</v>
+      </c>
+      <c r="AB13" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC13" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD13" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE13" s="53" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF13" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG13" s="53" t="n">
+        <v>32</v>
+      </c>
+      <c r="AH13" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI13" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ13" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK13" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL13" s="54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="L14" s="53" t="inlineStr">
+        <is>
+          <t>Estanteria Posterior</t>
+        </is>
+      </c>
+      <c r="M14" s="53" t="inlineStr"/>
+      <c r="N14" s="53" t="inlineStr"/>
+      <c r="O14" s="53" t="inlineStr"/>
+      <c r="P14" s="53" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q14" s="53" t="n">
+        <v>13</v>
+      </c>
+      <c r="R14" s="53" t="n">
+        <v>13</v>
+      </c>
+      <c r="S14" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="T14" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="V14" s="53" t="n">
+        <v>13</v>
+      </c>
+      <c r="W14" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="X14" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y14" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z14" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA14" s="53" t="n">
+        <v>13</v>
+      </c>
+      <c r="AB14" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC14" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD14" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE14" s="53" t="n">
+        <v>13</v>
+      </c>
+      <c r="AF14" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG14" s="53" t="n">
+        <v>12</v>
+      </c>
+      <c r="AH14" s="54" t="n">
+        <v>0.9230769230769231</v>
+      </c>
+      <c r="AI14" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ14" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK14" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL14" s="54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="L15" s="53" t="inlineStr">
+        <is>
+          <t>Interior 2</t>
+        </is>
+      </c>
+      <c r="M15" s="53" t="inlineStr"/>
+      <c r="N15" s="53" t="inlineStr"/>
+      <c r="O15" s="53" t="inlineStr"/>
+      <c r="P15" s="53" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q15" s="53" t="n">
+        <v>50</v>
+      </c>
+      <c r="R15" s="53" t="n">
+        <v>50</v>
+      </c>
+      <c r="S15" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="T15" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="U15" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="V15" s="53" t="n">
+        <v>50</v>
+      </c>
+      <c r="W15" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="X15" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y15" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z15" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA15" s="53" t="n">
+        <v>50</v>
+      </c>
+      <c r="AB15" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC15" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD15" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE15" s="53" t="n">
+        <v>50</v>
+      </c>
+      <c r="AF15" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AG15" s="53" t="n">
+        <v>47</v>
+      </c>
+      <c r="AH15" s="54" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="AI15" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ15" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK15" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL15" s="54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="L30" s="52" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="M30" s="52" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="N30" s="52" t="inlineStr">
+        <is>
+          <t>Hora_inicio</t>
+        </is>
+      </c>
+      <c r="O30" s="52" t="inlineStr">
+        <is>
+          <t>Hora_termino</t>
+        </is>
+      </c>
+      <c r="P30" s="52" t="inlineStr">
+        <is>
+          <t>Cámara</t>
+        </is>
+      </c>
+      <c r="Q30" s="52" t="inlineStr">
+        <is>
+          <t>Total Eventos</t>
+        </is>
+      </c>
+      <c r="R30" s="52" t="inlineStr">
+        <is>
+          <t>Eventos Registrados por el Sistema</t>
+        </is>
+      </c>
+      <c r="S30" s="52" t="inlineStr">
+        <is>
+          <t>% Eventos Registrados por el Sistema</t>
+        </is>
+      </c>
+      <c r="T30" s="52" t="inlineStr">
+        <is>
+          <t>Eventos NO Registrados (Manuales)</t>
+        </is>
+      </c>
+      <c r="U30" s="52" t="inlineStr">
+        <is>
+          <t>% Eventos NO Registrados (Manuales)</t>
+        </is>
+      </c>
+      <c r="V30" s="52" t="inlineStr">
+        <is>
+          <t>Eventos Correctos del Sistema</t>
+        </is>
+      </c>
+      <c r="W30" s="52" t="inlineStr">
+        <is>
+          <t>% Precisión de Eventos</t>
+        </is>
+      </c>
+      <c r="X30" s="52" t="inlineStr">
+        <is>
+          <t>% Eventos Correctos sobre Registrados</t>
+        </is>
+      </c>
+      <c r="Y30" s="52" t="inlineStr">
+        <is>
+          <t>Eventos Malos del Sistema</t>
+        </is>
+      </c>
+      <c r="Z30" s="52" t="inlineStr">
+        <is>
+          <t>% Eventos Malos sobre Total</t>
+        </is>
+      </c>
+      <c r="AA30" s="52" t="inlineStr">
+        <is>
+          <t>Cobertura Identity</t>
+        </is>
+      </c>
+      <c r="AB30" s="52" t="inlineStr">
+        <is>
+          <t>% Cobertura Identity</t>
+        </is>
+      </c>
+      <c r="AC30" s="52" t="inlineStr">
+        <is>
+          <t>Identity Unknown</t>
+        </is>
+      </c>
+      <c r="AD30" s="52" t="inlineStr">
+        <is>
+          <t>% Identity Unknown</t>
+        </is>
+      </c>
+      <c r="AE30" s="52" t="inlineStr">
+        <is>
+          <t>Cobertura Género</t>
+        </is>
+      </c>
+      <c r="AF30" s="52" t="inlineStr">
+        <is>
+          <t>% Cobertura Género</t>
+        </is>
+      </c>
+      <c r="AG30" s="52" t="inlineStr">
+        <is>
+          <t>Precisión de Género</t>
+        </is>
+      </c>
+      <c r="AH30" s="52" t="inlineStr">
+        <is>
+          <t>% Precisión de Género</t>
+        </is>
+      </c>
+      <c r="AI30" s="52" t="inlineStr">
+        <is>
+          <t>Cobertura Edad</t>
+        </is>
+      </c>
+      <c r="AJ30" s="52" t="inlineStr">
+        <is>
+          <t>% Cobertura Edad</t>
+        </is>
+      </c>
+      <c r="AK30" s="52" t="inlineStr">
+        <is>
+          <t>Precisión de Edad</t>
+        </is>
+      </c>
+      <c r="AL30" s="52" t="inlineStr">
+        <is>
+          <t>% Precisión de Edad</t>
+        </is>
+      </c>
+      <c r="AM30" s="52" t="inlineStr">
+        <is>
+          <t>Tipo_sensor</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="L31" s="53" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="M31" s="53" t="inlineStr"/>
+      <c r="N31" s="53" t="inlineStr"/>
+      <c r="O31" s="53" t="inlineStr"/>
+      <c r="P31" s="53" t="inlineStr"/>
+      <c r="Q31" s="53" t="n">
+        <v>626</v>
+      </c>
+      <c r="R31" s="53" t="n">
+        <v>617</v>
+      </c>
+      <c r="S31" s="54" t="n">
+        <v>0.9856230031948882</v>
+      </c>
+      <c r="T31" s="53" t="n">
+        <v>9</v>
+      </c>
+      <c r="U31" s="54" t="n">
+        <v>0.01437699680511182</v>
+      </c>
+      <c r="V31" s="53" t="n">
+        <v>605</v>
+      </c>
+      <c r="W31" s="54" t="n">
+        <v>0.9664536741214057</v>
+      </c>
+      <c r="X31" s="54" t="n">
+        <v>0.9805510534846029</v>
+      </c>
+      <c r="Y31" s="53" t="n">
+        <v>21</v>
+      </c>
+      <c r="Z31" s="54" t="n">
+        <v>0.03354632587859425</v>
+      </c>
+      <c r="AA31" s="53" t="n">
+        <v>418</v>
+      </c>
+      <c r="AB31" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC31" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD31" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE31" s="53" t="n">
+        <v>407</v>
+      </c>
+      <c r="AF31" s="54" t="n">
+        <v>0.9736842105263158</v>
+      </c>
+      <c r="AG31" s="53" t="n">
+        <v>389</v>
+      </c>
+      <c r="AH31" s="54" t="n">
+        <v>0.9557739557739557</v>
+      </c>
+      <c r="AI31" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ31" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK31" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL31" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM31" s="53" t="inlineStr"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -33238,9 +34496,391 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="X27:AB188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="27">
+      <c r="X27" s="52" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="Y27" s="52" t="inlineStr">
+        <is>
+          <t>Total eventos</t>
+        </is>
+      </c>
+      <c r="Z27" s="52" t="inlineStr">
+        <is>
+          <t>Eventos registrados por el sistema</t>
+        </is>
+      </c>
+      <c r="AA27" s="52" t="inlineStr">
+        <is>
+          <t>Precision de eventos</t>
+        </is>
+      </c>
+      <c r="AB27" s="52" t="inlineStr">
+        <is>
+          <t>Eventos no registrados por el sistema</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="X28" s="53" t="inlineStr">
+        <is>
+          <t>Entrada</t>
+        </is>
+      </c>
+      <c r="Y28" s="53" t="n">
+        <v>18</v>
+      </c>
+      <c r="Z28" s="53" t="n">
+        <v>18</v>
+      </c>
+      <c r="AA28" s="53" t="inlineStr">
+        <is>
+          <t>17 de 18 (94.44%)</t>
+        </is>
+      </c>
+      <c r="AB28" s="53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="X29" s="53" t="inlineStr">
+        <is>
+          <t>Exploracion 1</t>
+        </is>
+      </c>
+      <c r="Y29" s="53" t="n">
+        <v>30</v>
+      </c>
+      <c r="Z29" s="53" t="n">
+        <v>30</v>
+      </c>
+      <c r="AA29" s="53" t="inlineStr">
+        <is>
+          <t>30 de 30 (100.00%)</t>
+        </is>
+      </c>
+      <c r="AB29" s="53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="X30" s="53" t="inlineStr">
+        <is>
+          <t>Exterior 2</t>
+        </is>
+      </c>
+      <c r="Y30" s="53" t="n">
+        <v>105</v>
+      </c>
+      <c r="Z30" s="53" t="n">
+        <v>98</v>
+      </c>
+      <c r="AA30" s="53" t="inlineStr">
+        <is>
+          <t>98 de 105 (93.33%)</t>
+        </is>
+      </c>
+      <c r="AB30" s="53" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="X31" s="53" t="inlineStr">
+        <is>
+          <t>Exterior L</t>
+        </is>
+      </c>
+      <c r="Y31" s="53" t="n">
+        <v>103</v>
+      </c>
+      <c r="Z31" s="53" t="n">
+        <v>101</v>
+      </c>
+      <c r="AA31" s="53" t="inlineStr">
+        <is>
+          <t>100 de 103 (97.09%)</t>
+        </is>
+      </c>
+      <c r="AB31" s="53" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="X32" s="53" t="inlineStr">
+        <is>
+          <t>Vitrina Exterior</t>
+        </is>
+      </c>
+      <c r="Y32" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z32" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="AA32" s="53" t="inlineStr">
+        <is>
+          <t>6 de 6 (100.00%)</t>
+        </is>
+      </c>
+      <c r="AB32" s="53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="X33" s="53" t="inlineStr">
+        <is>
+          <t>Vitrina Interior</t>
+        </is>
+      </c>
+      <c r="Y33" s="53" t="n">
+        <v>14</v>
+      </c>
+      <c r="Z33" s="53" t="n">
+        <v>14</v>
+      </c>
+      <c r="AA33" s="53" t="inlineStr">
+        <is>
+          <t>14 de 14 (100.00%)</t>
+        </is>
+      </c>
+      <c r="AB33" s="53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="X80" s="52" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="Y80" s="52" t="inlineStr">
+        <is>
+          <t>Total eventos</t>
+        </is>
+      </c>
+      <c r="Z80" s="52" t="inlineStr">
+        <is>
+          <t>Eventos registrados por el sistema</t>
+        </is>
+      </c>
+      <c r="AA80" s="52" t="inlineStr">
+        <is>
+          <t>Precision de eventos</t>
+        </is>
+      </c>
+      <c r="AB80" s="52" t="inlineStr">
+        <is>
+          <t>Eventos no registrados por el sistema</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="X81" s="53" t="inlineStr">
+        <is>
+          <t>Interior 1</t>
+        </is>
+      </c>
+      <c r="Y81" s="53" t="n">
+        <v>16</v>
+      </c>
+      <c r="Z81" s="53" t="n">
+        <v>16</v>
+      </c>
+      <c r="AA81" s="53" t="inlineStr">
+        <is>
+          <t>16 de 16 (100.00%)</t>
+        </is>
+      </c>
+      <c r="AB81" s="53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="X133" s="52" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="Y133" s="52" t="inlineStr">
+        <is>
+          <t>Total eventos</t>
+        </is>
+      </c>
+      <c r="Z133" s="52" t="inlineStr">
+        <is>
+          <t>Eventos registrados por el sistema</t>
+        </is>
+      </c>
+      <c r="AA133" s="52" t="inlineStr">
+        <is>
+          <t>Precision de eventos</t>
+        </is>
+      </c>
+      <c r="AB133" s="52" t="inlineStr">
+        <is>
+          <t>Eventos no registrados por el sistema</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="X134" s="53" t="inlineStr">
+        <is>
+          <t>Caja</t>
+        </is>
+      </c>
+      <c r="Y134" s="53" t="n">
+        <v>77</v>
+      </c>
+      <c r="Z134" s="53" t="n">
+        <v>77</v>
+      </c>
+      <c r="AA134" s="53" t="inlineStr">
+        <is>
+          <t>77 de 77 (100.00%)</t>
+        </is>
+      </c>
+      <c r="AB134" s="53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="X135" s="53" t="inlineStr">
+        <is>
+          <t>Estanteria Principal</t>
+        </is>
+      </c>
+      <c r="Y135" s="53" t="n">
+        <v>106</v>
+      </c>
+      <c r="Z135" s="53" t="n">
+        <v>106</v>
+      </c>
+      <c r="AA135" s="53" t="inlineStr">
+        <is>
+          <t>100 de 106 (94.34%)</t>
+        </is>
+      </c>
+      <c r="AB135" s="53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="X136" s="53" t="inlineStr">
+        <is>
+          <t>Exploracion 2</t>
+        </is>
+      </c>
+      <c r="Y136" s="53" t="n">
+        <v>56</v>
+      </c>
+      <c r="Z136" s="53" t="n">
+        <v>56</v>
+      </c>
+      <c r="AA136" s="53" t="inlineStr">
+        <is>
+          <t>53 de 56 (94.64%)</t>
+        </is>
+      </c>
+      <c r="AB136" s="53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="X137" s="53" t="inlineStr">
+        <is>
+          <t>Exploracion 3</t>
+        </is>
+      </c>
+      <c r="Y137" s="53" t="n">
+        <v>32</v>
+      </c>
+      <c r="Z137" s="53" t="n">
+        <v>32</v>
+      </c>
+      <c r="AA137" s="53" t="inlineStr">
+        <is>
+          <t>31 de 32 (96.88%)</t>
+        </is>
+      </c>
+      <c r="AB137" s="53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="X186" s="52" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="Y186" s="52" t="inlineStr">
+        <is>
+          <t>Total eventos</t>
+        </is>
+      </c>
+      <c r="Z186" s="52" t="inlineStr">
+        <is>
+          <t>Eventos registrados por el sistema</t>
+        </is>
+      </c>
+      <c r="AA186" s="52" t="inlineStr">
+        <is>
+          <t>Precision de eventos</t>
+        </is>
+      </c>
+      <c r="AB186" s="52" t="inlineStr">
+        <is>
+          <t>Eventos no registrados por el sistema</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="X187" s="53" t="inlineStr">
+        <is>
+          <t>Estanteria Posterior</t>
+        </is>
+      </c>
+      <c r="Y187" s="53" t="n">
+        <v>13</v>
+      </c>
+      <c r="Z187" s="53" t="n">
+        <v>13</v>
+      </c>
+      <c r="AA187" s="53" t="inlineStr">
+        <is>
+          <t>13 de 13 (100.00%)</t>
+        </is>
+      </c>
+      <c r="AB187" s="53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="X188" s="53" t="inlineStr">
+        <is>
+          <t>Interior 2</t>
+        </is>
+      </c>
+      <c r="Y188" s="53" t="n">
+        <v>50</v>
+      </c>
+      <c r="Z188" s="53" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA188" s="53" t="inlineStr">
+        <is>
+          <t>50 de 50 (100.00%)</t>
+        </is>
+      </c>
+      <c r="AB188" s="53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -33252,9 +34892,634 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="L2:P303"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="2">
+      <c r="L2" s="52" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="M2" s="52" t="inlineStr">
+        <is>
+          <t>Total eventos</t>
+        </is>
+      </c>
+      <c r="N2" s="52" t="inlineStr">
+        <is>
+          <t>Eventos registrados por el sistema</t>
+        </is>
+      </c>
+      <c r="O2" s="52" t="inlineStr">
+        <is>
+          <t>Precision de eventos</t>
+        </is>
+      </c>
+      <c r="P2" s="52" t="inlineStr">
+        <is>
+          <t>Eventos no registrados por el sistema</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="L3" s="53" t="inlineStr">
+        <is>
+          <t>Entrada</t>
+        </is>
+      </c>
+      <c r="M3" s="53" t="n">
+        <v>18</v>
+      </c>
+      <c r="N3" s="53" t="n">
+        <v>18</v>
+      </c>
+      <c r="O3" s="53" t="inlineStr">
+        <is>
+          <t>17 de 18 (94.44%)</t>
+        </is>
+      </c>
+      <c r="P3" s="53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="L27" s="52" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="M27" s="52" t="inlineStr">
+        <is>
+          <t>Total eventos</t>
+        </is>
+      </c>
+      <c r="N27" s="52" t="inlineStr">
+        <is>
+          <t>Eventos registrados por el sistema</t>
+        </is>
+      </c>
+      <c r="O27" s="52" t="inlineStr">
+        <is>
+          <t>Precision de eventos</t>
+        </is>
+      </c>
+      <c r="P27" s="52" t="inlineStr">
+        <is>
+          <t>Eventos no registrados por el sistema</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="L28" s="53" t="inlineStr">
+        <is>
+          <t>Exploracion 1</t>
+        </is>
+      </c>
+      <c r="M28" s="53" t="n">
+        <v>30</v>
+      </c>
+      <c r="N28" s="53" t="n">
+        <v>30</v>
+      </c>
+      <c r="O28" s="53" t="inlineStr">
+        <is>
+          <t>30 de 30 (100.00%)</t>
+        </is>
+      </c>
+      <c r="P28" s="53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="L52" s="52" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="M52" s="52" t="inlineStr">
+        <is>
+          <t>Total eventos</t>
+        </is>
+      </c>
+      <c r="N52" s="52" t="inlineStr">
+        <is>
+          <t>Eventos registrados por el sistema</t>
+        </is>
+      </c>
+      <c r="O52" s="52" t="inlineStr">
+        <is>
+          <t>Precision de eventos</t>
+        </is>
+      </c>
+      <c r="P52" s="52" t="inlineStr">
+        <is>
+          <t>Eventos no registrados por el sistema</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="L53" s="53" t="inlineStr">
+        <is>
+          <t>Exterior 2</t>
+        </is>
+      </c>
+      <c r="M53" s="53" t="n">
+        <v>105</v>
+      </c>
+      <c r="N53" s="53" t="n">
+        <v>98</v>
+      </c>
+      <c r="O53" s="53" t="inlineStr">
+        <is>
+          <t>98 de 105 (93.33%)</t>
+        </is>
+      </c>
+      <c r="P53" s="53" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="L77" s="52" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="M77" s="52" t="inlineStr">
+        <is>
+          <t>Total eventos</t>
+        </is>
+      </c>
+      <c r="N77" s="52" t="inlineStr">
+        <is>
+          <t>Eventos registrados por el sistema</t>
+        </is>
+      </c>
+      <c r="O77" s="52" t="inlineStr">
+        <is>
+          <t>Precision de eventos</t>
+        </is>
+      </c>
+      <c r="P77" s="52" t="inlineStr">
+        <is>
+          <t>Eventos no registrados por el sistema</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="L78" s="53" t="inlineStr">
+        <is>
+          <t>Exterior L</t>
+        </is>
+      </c>
+      <c r="M78" s="53" t="n">
+        <v>103</v>
+      </c>
+      <c r="N78" s="53" t="n">
+        <v>101</v>
+      </c>
+      <c r="O78" s="53" t="inlineStr">
+        <is>
+          <t>100 de 103 (97.09%)</t>
+        </is>
+      </c>
+      <c r="P78" s="53" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="L102" s="52" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="M102" s="52" t="inlineStr">
+        <is>
+          <t>Total eventos</t>
+        </is>
+      </c>
+      <c r="N102" s="52" t="inlineStr">
+        <is>
+          <t>Eventos registrados por el sistema</t>
+        </is>
+      </c>
+      <c r="O102" s="52" t="inlineStr">
+        <is>
+          <t>Precision de eventos</t>
+        </is>
+      </c>
+      <c r="P102" s="52" t="inlineStr">
+        <is>
+          <t>Eventos no registrados por el sistema</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="L103" s="53" t="inlineStr">
+        <is>
+          <t>Vitrina Exterior</t>
+        </is>
+      </c>
+      <c r="M103" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="N103" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="O103" s="53" t="inlineStr">
+        <is>
+          <t>6 de 6 (100.00%)</t>
+        </is>
+      </c>
+      <c r="P103" s="53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="L127" s="52" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="M127" s="52" t="inlineStr">
+        <is>
+          <t>Total eventos</t>
+        </is>
+      </c>
+      <c r="N127" s="52" t="inlineStr">
+        <is>
+          <t>Eventos registrados por el sistema</t>
+        </is>
+      </c>
+      <c r="O127" s="52" t="inlineStr">
+        <is>
+          <t>Precision de eventos</t>
+        </is>
+      </c>
+      <c r="P127" s="52" t="inlineStr">
+        <is>
+          <t>Eventos no registrados por el sistema</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="L128" s="53" t="inlineStr">
+        <is>
+          <t>Vitrina Interior</t>
+        </is>
+      </c>
+      <c r="M128" s="53" t="n">
+        <v>14</v>
+      </c>
+      <c r="N128" s="53" t="n">
+        <v>14</v>
+      </c>
+      <c r="O128" s="53" t="inlineStr">
+        <is>
+          <t>14 de 14 (100.00%)</t>
+        </is>
+      </c>
+      <c r="P128" s="53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="L152" s="52" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="M152" s="52" t="inlineStr">
+        <is>
+          <t>Total eventos</t>
+        </is>
+      </c>
+      <c r="N152" s="52" t="inlineStr">
+        <is>
+          <t>Eventos registrados por el sistema</t>
+        </is>
+      </c>
+      <c r="O152" s="52" t="inlineStr">
+        <is>
+          <t>Precision de eventos</t>
+        </is>
+      </c>
+      <c r="P152" s="52" t="inlineStr">
+        <is>
+          <t>Eventos no registrados por el sistema</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="L153" s="53" t="inlineStr">
+        <is>
+          <t>Interior 1</t>
+        </is>
+      </c>
+      <c r="M153" s="53" t="n">
+        <v>16</v>
+      </c>
+      <c r="N153" s="53" t="n">
+        <v>16</v>
+      </c>
+      <c r="O153" s="53" t="inlineStr">
+        <is>
+          <t>16 de 16 (100.00%)</t>
+        </is>
+      </c>
+      <c r="P153" s="53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="L177" s="52" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="M177" s="52" t="inlineStr">
+        <is>
+          <t>Total eventos</t>
+        </is>
+      </c>
+      <c r="N177" s="52" t="inlineStr">
+        <is>
+          <t>Eventos registrados por el sistema</t>
+        </is>
+      </c>
+      <c r="O177" s="52" t="inlineStr">
+        <is>
+          <t>Precision de eventos</t>
+        </is>
+      </c>
+      <c r="P177" s="52" t="inlineStr">
+        <is>
+          <t>Eventos no registrados por el sistema</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="L178" s="53" t="inlineStr">
+        <is>
+          <t>Caja</t>
+        </is>
+      </c>
+      <c r="M178" s="53" t="n">
+        <v>77</v>
+      </c>
+      <c r="N178" s="53" t="n">
+        <v>77</v>
+      </c>
+      <c r="O178" s="53" t="inlineStr">
+        <is>
+          <t>77 de 77 (100.00%)</t>
+        </is>
+      </c>
+      <c r="P178" s="53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="L202" s="52" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="M202" s="52" t="inlineStr">
+        <is>
+          <t>Total eventos</t>
+        </is>
+      </c>
+      <c r="N202" s="52" t="inlineStr">
+        <is>
+          <t>Eventos registrados por el sistema</t>
+        </is>
+      </c>
+      <c r="O202" s="52" t="inlineStr">
+        <is>
+          <t>Precision de eventos</t>
+        </is>
+      </c>
+      <c r="P202" s="52" t="inlineStr">
+        <is>
+          <t>Eventos no registrados por el sistema</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="L203" s="53" t="inlineStr">
+        <is>
+          <t>Estanteria Principal</t>
+        </is>
+      </c>
+      <c r="M203" s="53" t="n">
+        <v>106</v>
+      </c>
+      <c r="N203" s="53" t="n">
+        <v>106</v>
+      </c>
+      <c r="O203" s="53" t="inlineStr">
+        <is>
+          <t>100 de 106 (94.34%)</t>
+        </is>
+      </c>
+      <c r="P203" s="53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="L227" s="52" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="M227" s="52" t="inlineStr">
+        <is>
+          <t>Total eventos</t>
+        </is>
+      </c>
+      <c r="N227" s="52" t="inlineStr">
+        <is>
+          <t>Eventos registrados por el sistema</t>
+        </is>
+      </c>
+      <c r="O227" s="52" t="inlineStr">
+        <is>
+          <t>Precision de eventos</t>
+        </is>
+      </c>
+      <c r="P227" s="52" t="inlineStr">
+        <is>
+          <t>Eventos no registrados por el sistema</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="L228" s="53" t="inlineStr">
+        <is>
+          <t>Exploracion 2</t>
+        </is>
+      </c>
+      <c r="M228" s="53" t="n">
+        <v>56</v>
+      </c>
+      <c r="N228" s="53" t="n">
+        <v>56</v>
+      </c>
+      <c r="O228" s="53" t="inlineStr">
+        <is>
+          <t>53 de 56 (94.64%)</t>
+        </is>
+      </c>
+      <c r="P228" s="53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="L252" s="52" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="M252" s="52" t="inlineStr">
+        <is>
+          <t>Total eventos</t>
+        </is>
+      </c>
+      <c r="N252" s="52" t="inlineStr">
+        <is>
+          <t>Eventos registrados por el sistema</t>
+        </is>
+      </c>
+      <c r="O252" s="52" t="inlineStr">
+        <is>
+          <t>Precision de eventos</t>
+        </is>
+      </c>
+      <c r="P252" s="52" t="inlineStr">
+        <is>
+          <t>Eventos no registrados por el sistema</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="L253" s="53" t="inlineStr">
+        <is>
+          <t>Exploracion 3</t>
+        </is>
+      </c>
+      <c r="M253" s="53" t="n">
+        <v>32</v>
+      </c>
+      <c r="N253" s="53" t="n">
+        <v>32</v>
+      </c>
+      <c r="O253" s="53" t="inlineStr">
+        <is>
+          <t>31 de 32 (96.88%)</t>
+        </is>
+      </c>
+      <c r="P253" s="53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="L277" s="52" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="M277" s="52" t="inlineStr">
+        <is>
+          <t>Total eventos</t>
+        </is>
+      </c>
+      <c r="N277" s="52" t="inlineStr">
+        <is>
+          <t>Eventos registrados por el sistema</t>
+        </is>
+      </c>
+      <c r="O277" s="52" t="inlineStr">
+        <is>
+          <t>Precision de eventos</t>
+        </is>
+      </c>
+      <c r="P277" s="52" t="inlineStr">
+        <is>
+          <t>Eventos no registrados por el sistema</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="L278" s="53" t="inlineStr">
+        <is>
+          <t>Estanteria Posterior</t>
+        </is>
+      </c>
+      <c r="M278" s="53" t="n">
+        <v>13</v>
+      </c>
+      <c r="N278" s="53" t="n">
+        <v>13</v>
+      </c>
+      <c r="O278" s="53" t="inlineStr">
+        <is>
+          <t>13 de 13 (100.00%)</t>
+        </is>
+      </c>
+      <c r="P278" s="53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="L302" s="52" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="M302" s="52" t="inlineStr">
+        <is>
+          <t>Total eventos</t>
+        </is>
+      </c>
+      <c r="N302" s="52" t="inlineStr">
+        <is>
+          <t>Eventos registrados por el sistema</t>
+        </is>
+      </c>
+      <c r="O302" s="52" t="inlineStr">
+        <is>
+          <t>Precision de eventos</t>
+        </is>
+      </c>
+      <c r="P302" s="52" t="inlineStr">
+        <is>
+          <t>Eventos no registrados por el sistema</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="L303" s="53" t="inlineStr">
+        <is>
+          <t>Interior 2</t>
+        </is>
+      </c>
+      <c r="M303" s="53" t="n">
+        <v>50</v>
+      </c>
+      <c r="N303" s="53" t="n">
+        <v>50</v>
+      </c>
+      <c r="O303" s="53" t="inlineStr">
+        <is>
+          <t>50 de 50 (100.00%)</t>
+        </is>
+      </c>
+      <c r="P303" s="53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -33266,9 +35531,466 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="L2:O279"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="2">
+      <c r="L2" s="52" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="M2" s="52" t="inlineStr">
+        <is>
+          <t>Eventos Registrados por el Sistema</t>
+        </is>
+      </c>
+      <c r="N2" s="52" t="inlineStr">
+        <is>
+          <t>Identity Unknown</t>
+        </is>
+      </c>
+      <c r="O2" s="52" t="inlineStr">
+        <is>
+          <t>% Identity Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="L3" s="53" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="M3" s="53" t="n">
+        <v>617</v>
+      </c>
+      <c r="N3" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="L28" s="52" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="M28" s="52" t="inlineStr">
+        <is>
+          <t>Eventos Registrados por el Sistema</t>
+        </is>
+      </c>
+      <c r="N28" s="52" t="inlineStr">
+        <is>
+          <t>Identity Unknown</t>
+        </is>
+      </c>
+      <c r="O28" s="52" t="inlineStr">
+        <is>
+          <t>% Identity Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="L29" s="53" t="inlineStr">
+        <is>
+          <t>Entrada</t>
+        </is>
+      </c>
+      <c r="M29" s="53" t="n">
+        <v>18</v>
+      </c>
+      <c r="N29" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" s="54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="L53" s="52" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="M53" s="52" t="inlineStr">
+        <is>
+          <t>Eventos Registrados por el Sistema</t>
+        </is>
+      </c>
+      <c r="N53" s="52" t="inlineStr">
+        <is>
+          <t>Identity Unknown</t>
+        </is>
+      </c>
+      <c r="O53" s="52" t="inlineStr">
+        <is>
+          <t>% Identity Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="L54" s="53" t="inlineStr">
+        <is>
+          <t>Exploracion 1</t>
+        </is>
+      </c>
+      <c r="M54" s="53" t="n">
+        <v>30</v>
+      </c>
+      <c r="N54" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="O54" s="54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="L78" s="52" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="M78" s="52" t="inlineStr">
+        <is>
+          <t>Eventos Registrados por el Sistema</t>
+        </is>
+      </c>
+      <c r="N78" s="52" t="inlineStr">
+        <is>
+          <t>Identity Unknown</t>
+        </is>
+      </c>
+      <c r="O78" s="52" t="inlineStr">
+        <is>
+          <t>% Identity Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="L79" s="53" t="inlineStr">
+        <is>
+          <t>Vitrina Exterior</t>
+        </is>
+      </c>
+      <c r="M79" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="N79" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="O79" s="54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="L103" s="52" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="M103" s="52" t="inlineStr">
+        <is>
+          <t>Eventos Registrados por el Sistema</t>
+        </is>
+      </c>
+      <c r="N103" s="52" t="inlineStr">
+        <is>
+          <t>Identity Unknown</t>
+        </is>
+      </c>
+      <c r="O103" s="52" t="inlineStr">
+        <is>
+          <t>% Identity Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="L104" s="53" t="inlineStr">
+        <is>
+          <t>Vitrina Interior</t>
+        </is>
+      </c>
+      <c r="M104" s="53" t="n">
+        <v>14</v>
+      </c>
+      <c r="N104" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="O104" s="54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="L128" s="52" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="M128" s="52" t="inlineStr">
+        <is>
+          <t>Eventos Registrados por el Sistema</t>
+        </is>
+      </c>
+      <c r="N128" s="52" t="inlineStr">
+        <is>
+          <t>Identity Unknown</t>
+        </is>
+      </c>
+      <c r="O128" s="52" t="inlineStr">
+        <is>
+          <t>% Identity Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="L129" s="53" t="inlineStr">
+        <is>
+          <t>Interior 1</t>
+        </is>
+      </c>
+      <c r="M129" s="53" t="n">
+        <v>16</v>
+      </c>
+      <c r="N129" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="O129" s="54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="L153" s="52" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="M153" s="52" t="inlineStr">
+        <is>
+          <t>Eventos Registrados por el Sistema</t>
+        </is>
+      </c>
+      <c r="N153" s="52" t="inlineStr">
+        <is>
+          <t>Identity Unknown</t>
+        </is>
+      </c>
+      <c r="O153" s="52" t="inlineStr">
+        <is>
+          <t>% Identity Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="L154" s="53" t="inlineStr">
+        <is>
+          <t>Caja</t>
+        </is>
+      </c>
+      <c r="M154" s="53" t="n">
+        <v>77</v>
+      </c>
+      <c r="N154" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="O154" s="54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="L178" s="52" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="M178" s="52" t="inlineStr">
+        <is>
+          <t>Eventos Registrados por el Sistema</t>
+        </is>
+      </c>
+      <c r="N178" s="52" t="inlineStr">
+        <is>
+          <t>Identity Unknown</t>
+        </is>
+      </c>
+      <c r="O178" s="52" t="inlineStr">
+        <is>
+          <t>% Identity Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="L179" s="53" t="inlineStr">
+        <is>
+          <t>Estanteria Principal</t>
+        </is>
+      </c>
+      <c r="M179" s="53" t="n">
+        <v>106</v>
+      </c>
+      <c r="N179" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="O179" s="54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="L203" s="52" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="M203" s="52" t="inlineStr">
+        <is>
+          <t>Eventos Registrados por el Sistema</t>
+        </is>
+      </c>
+      <c r="N203" s="52" t="inlineStr">
+        <is>
+          <t>Identity Unknown</t>
+        </is>
+      </c>
+      <c r="O203" s="52" t="inlineStr">
+        <is>
+          <t>% Identity Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="L204" s="53" t="inlineStr">
+        <is>
+          <t>Exploracion 2</t>
+        </is>
+      </c>
+      <c r="M204" s="53" t="n">
+        <v>56</v>
+      </c>
+      <c r="N204" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="O204" s="54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="L228" s="52" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="M228" s="52" t="inlineStr">
+        <is>
+          <t>Eventos Registrados por el Sistema</t>
+        </is>
+      </c>
+      <c r="N228" s="52" t="inlineStr">
+        <is>
+          <t>Identity Unknown</t>
+        </is>
+      </c>
+      <c r="O228" s="52" t="inlineStr">
+        <is>
+          <t>% Identity Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="L229" s="53" t="inlineStr">
+        <is>
+          <t>Exploracion 3</t>
+        </is>
+      </c>
+      <c r="M229" s="53" t="n">
+        <v>32</v>
+      </c>
+      <c r="N229" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="O229" s="54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="L253" s="52" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="M253" s="52" t="inlineStr">
+        <is>
+          <t>Eventos Registrados por el Sistema</t>
+        </is>
+      </c>
+      <c r="N253" s="52" t="inlineStr">
+        <is>
+          <t>Identity Unknown</t>
+        </is>
+      </c>
+      <c r="O253" s="52" t="inlineStr">
+        <is>
+          <t>% Identity Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="L254" s="53" t="inlineStr">
+        <is>
+          <t>Estanteria Posterior</t>
+        </is>
+      </c>
+      <c r="M254" s="53" t="n">
+        <v>13</v>
+      </c>
+      <c r="N254" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="O254" s="54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="L278" s="52" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="M278" s="52" t="inlineStr">
+        <is>
+          <t>Eventos Registrados por el Sistema</t>
+        </is>
+      </c>
+      <c r="N278" s="52" t="inlineStr">
+        <is>
+          <t>Identity Unknown</t>
+        </is>
+      </c>
+      <c r="O278" s="52" t="inlineStr">
+        <is>
+          <t>% Identity Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="L279" s="53" t="inlineStr">
+        <is>
+          <t>Interior 2</t>
+        </is>
+      </c>
+      <c r="M279" s="53" t="n">
+        <v>50</v>
+      </c>
+      <c r="N279" s="53" t="n">
+        <v>0</v>
+      </c>
+      <c r="O279" s="54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>

</xml_diff>